<commit_message>
Update test cases spreadsheet with new test scenarios
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test_automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/274008f7bd52386a/Desktop/IT23377158/test_automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6093456D-2646-4D6B-8FF5-3CCDE59B9837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{6093456D-2646-4D6B-8FF5-3CCDE59B9837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F48009F8-F73F-4E28-8756-AFC3AFFE6BDD}"/>
   <bookViews>
-    <workbookView xWindow="7728" yWindow="732" windowWidth="14328" windowHeight="8880" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" Test cases" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="287">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -647,13 +647,247 @@
   </si>
   <si>
     <t>pdf 3ක්ම ඕනේ වෙන්න.</t>
+  </si>
+  <si>
+    <t>Question forms</t>
+  </si>
+  <si>
+    <t>Command forms</t>
+  </si>
+  <si>
+    <t>Greetings</t>
+  </si>
+  <si>
+    <t>Requests</t>
+  </si>
+  <si>
+    <t>Responses</t>
+  </si>
+  <si>
+    <t>Repeated Words</t>
+  </si>
+  <si>
+    <t>Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Isolated English Word Insertions in Singlish</t>
+  </si>
+  <si>
+    <t>Multi-Word English Phrases in Singlish</t>
+  </si>
+  <si>
+    <t>English Digital Terms in Singlish</t>
+  </si>
+  <si>
+    <t>Platform/App Names in Singlish</t>
+  </si>
+  <si>
+    <t>English Abbreviations/Acronyms in Singlish</t>
+  </si>
+  <si>
+    <t>English Clipped Forms in Singlish</t>
+  </si>
+  <si>
+    <t>Place Names Embedded in Singlish</t>
+  </si>
+  <si>
+    <t>Person Names Embedded in Singlish</t>
+  </si>
+  <si>
+    <t>Inputs with Numbers and Numeric Suffixes</t>
+  </si>
+  <si>
+    <t>Inputs with Currency</t>
+  </si>
+  <si>
+    <t>Inputs with Time Formats</t>
+  </si>
+  <si>
+    <t>Inputs with Dates</t>
+  </si>
+  <si>
+    <t>Inputs with Unit of Measurements</t>
+  </si>
+  <si>
+    <t>Inputs with Slang and Casual Phrasing</t>
+  </si>
+  <si>
+    <t>Online Identifiers in Singlish</t>
+  </si>
+  <si>
+    <t>Inputs Containing Emojis</t>
+  </si>
+  <si>
+    <t>Greetings; Inputs with Dates; Place Names Embedded in Singlish; Isolated English Word Insertions in Singlish; Question forms</t>
+  </si>
+  <si>
+    <t>Question forms; Inputs with Currency; Place Names Embedded in Singlish; Isolated English Word Insertions in Singlish</t>
+  </si>
+  <si>
+    <t>Singlish Input Types Covered</t>
+  </si>
+  <si>
+    <t>Rationale: The input asks “why did you do that?” and ends with a question mark, so it is a question form.</t>
+  </si>
+  <si>
+    <t>Rationale: The input asks whether notes can be sent if the person attends lectures, using “ewanawada?” and a question mark.</t>
+  </si>
+  <si>
+    <t>Rationale: The input gives an instruction to bring mangoes when coming; the command verb “genna” shows a command form.</t>
+  </si>
+  <si>
+    <t>Rationale: The input instructs the user to go to a website and check it; the verb “balanna” indicates a command.</t>
+  </si>
+  <si>
+    <t>Rationale: The phrase “suba udasanak wewa!” is used to wish someone a good morning.</t>
+  </si>
+  <si>
+    <t>Rationale: The phrase “theruwan saranai!” is a common Sinhala blessing/greeting.</t>
+  </si>
+  <si>
+    <t>Rationale: The input politely asks for money as a loan using “anee” and “denna,” so it is a request.</t>
+  </si>
+  <si>
+    <t>Rationale: The word “puluwannam” means “if possible,” and the sentence asks the person to come tomorrow, making it a request.</t>
+  </si>
+  <si>
+    <t>Rationale: The sentence gives a reply/explanation about being sick yesterday, so it is used as a response.</t>
+  </si>
+  <si>
+    <t>Rationale: The input starts with “nope” and then says “mama kiyannam,” showing a reply/response.</t>
+  </si>
+  <si>
+    <t>Rationale: The word “onna” is repeated twice at the beginning, so this tests repeated words.</t>
+  </si>
+  <si>
+    <t>Rationale: The word “hari” is repeated twice, so this belongs to repeated words.</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses several punctuation marks, including “!!!” and “?”, so it tests punctuation handling.</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses an ellipsis “...” between two parts of the sentence, so it tests punctuation marks.</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard continuous chat-style spelling without proper spacing, so it tests romanization/spelling variation.</t>
+  </si>
+  <si>
+    <t>Rationale: The shortened form “ht” is used instead of “heta,” so this tests Romanization/spelling variants.</t>
+  </si>
+  <si>
+    <t>Rationale: The English word “gym” is inserted into a Singlish sentence.</t>
+  </si>
+  <si>
+    <t>Rationale: The English word “shop” is inserted into a Singlish sentence.</t>
+  </si>
+  <si>
+    <t>Rationale: The phrase “No way” contains two consecutive English words inside the Singlish sentence.</t>
+  </si>
+  <si>
+    <t>Rationale: The phrase “second half” is a multi-word English phrase inserted within the Singlish sentence.</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains digital terms such as “screenshot,” “USB,” and “copy.”</t>
+  </si>
+  <si>
+    <t>Rationale: The word “username” is a digital/account-related English term used in the Singlish sentence.</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the platform/app name “Facebook.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the platform name “linkedin.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the abbreviations/acronyms “CV” and “HR.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the abbreviations/acronyms “ID” and “PDF.”</t>
+  </si>
+  <si>
+    <t>Rationale: The word “lec” is a clipped form of “lecture.”</t>
+  </si>
+  <si>
+    <t>Rationale: The word “doc” is a clipped form of “document.”</t>
+  </si>
+  <si>
+    <t>Rationale: The place name “Colombo” is embedded in the Singlish sentence.</t>
+  </si>
+  <si>
+    <t>Rationale: The place name “Galle” appears in the input as “Galleta,” meaning “to Galle.”</t>
+  </si>
+  <si>
+    <t>Rationale: The person names “Kavindii” and “Tharakai” are embedded in the Singlish sentence.</t>
+  </si>
+  <si>
+    <t>Rationale: The person name “Kasun” is embedded in the input as “Kasunta.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the number with suffix “2k,” meaning “2ක්.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the number with suffix “3kma,” meaning “3ක්ම.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the currency abbreviation “lkr” with the amount “350.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains “Rs. 1200k,” which combines a currency value with a Sinhala-style numeric suffix.</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the time format “8.30ta,” meaning “at 8.30.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the time format “6:45PM.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the date expression “March 10.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the date expression “April 20.”</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the measurement “ml 500,” so it tests units of measurement.</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the measurement “kg 10k,” so it tests units of measurement.</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses casual/slang wording such as “ado,” so it tests slang and casual phrasing.</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses casual/slang words such as “ado” and “uba,” so it tests slang and casual phrasing.</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the email address “test123@yahoo.com,” which is an online identifier.</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the website address “www.example.lk,” which is an online identifier.</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the emoji “😩,” so it tests inputs containing emojis.</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the emoji “🎉,” so it tests inputs containing emojis.</t>
+  </si>
+  <si>
+    <t>Evidence: “Good morning” is a greeting; “March 15” is a date; “Mirissa” is a place name; “beach trip” and “cancel” include English words; and “karamuda?” makes it a question.</t>
+  </si>
+  <si>
+    <t>Evidence: “athida?” makes the sentence a question; “Rs. 500k” is a currency value; “Galle” is a place name; and “bus” is an isolated English word inside Singlish.</t>
+  </si>
+  <si>
+    <t>Evidence or rationale for the input type covered</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -667,6 +901,11 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -707,10 +946,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -721,9 +961,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{75BC6F1A-8916-4C8A-8D7B-0ED1171B10C6}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1001,7 +1255,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="49.95" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1010,10 +1264,11 @@
     <col min="4" max="4" width="36.88671875" customWidth="1"/>
     <col min="5" max="5" width="71.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="8" width="12.33203125" customWidth="1"/>
+    <col min="7" max="7" width="104.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="36.6" customHeight="1">
+    <row r="1" spans="1:8" ht="36.6" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1032,8 +1287,14 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G1" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="49.95" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1052,8 +1313,14 @@
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G2" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="49.95" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -1072,8 +1339,14 @@
       <c r="F3" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G3" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="49.95" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1092,8 +1365,14 @@
       <c r="F4" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="58.8" customHeight="1">
+      <c r="G4" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="58.8" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -1112,8 +1391,14 @@
       <c r="F5" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G5" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="49.95" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -1132,8 +1417,14 @@
       <c r="F6" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G6" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="49.95" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -1152,8 +1443,14 @@
       <c r="F7" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G7" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="49.95" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
@@ -1172,8 +1469,14 @@
       <c r="F8" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G8" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="49.95" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
@@ -1192,8 +1495,14 @@
       <c r="F9" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G9" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="49.95" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -1212,8 +1521,14 @@
       <c r="F10" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G10" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="49.95" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>22</v>
       </c>
@@ -1232,8 +1547,14 @@
       <c r="F11" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G11" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="49.95" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>23</v>
       </c>
@@ -1252,8 +1573,14 @@
       <c r="F12" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G12" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="49.95" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>24</v>
       </c>
@@ -1272,8 +1599,14 @@
       <c r="F13" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G13" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="49.95" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
@@ -1292,8 +1625,14 @@
       <c r="F14" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G14" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="49.95" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>28</v>
       </c>
@@ -1312,8 +1651,14 @@
       <c r="F15" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G15" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="49.95" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
@@ -1332,8 +1677,14 @@
       <c r="F16" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G16" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="49.95" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>32</v>
       </c>
@@ -1352,8 +1703,14 @@
       <c r="F17" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G17" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="49.95" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>33</v>
       </c>
@@ -1372,8 +1729,14 @@
       <c r="F18" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G18" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="49.95" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>34</v>
       </c>
@@ -1392,8 +1755,14 @@
       <c r="F19" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G19" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="49.95" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>35</v>
       </c>
@@ -1412,8 +1781,14 @@
       <c r="F20" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G20" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="49.95" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>36</v>
       </c>
@@ -1432,8 +1807,14 @@
       <c r="F21" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G21" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="49.95" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>37</v>
       </c>
@@ -1452,8 +1833,14 @@
       <c r="F22" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G22" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="49.95" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>38</v>
       </c>
@@ -1472,8 +1859,14 @@
       <c r="F23" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G23" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="49.95" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>39</v>
       </c>
@@ -1492,8 +1885,14 @@
       <c r="F24" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G24" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="49.95" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>40</v>
       </c>
@@ -1512,8 +1911,14 @@
       <c r="F25" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G25" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="49.95" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>42</v>
       </c>
@@ -1532,8 +1937,14 @@
       <c r="F26" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G26" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="49.95" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>45</v>
       </c>
@@ -1552,8 +1963,14 @@
       <c r="F27" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G27" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="49.95" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>48</v>
       </c>
@@ -1572,8 +1989,14 @@
       <c r="F28" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G28" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="49.95" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>51</v>
       </c>
@@ -1592,8 +2015,14 @@
       <c r="F29" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G29" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="49.95" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>54</v>
       </c>
@@ -1612,8 +2041,14 @@
       <c r="F30" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G30" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="49.95" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>55</v>
       </c>
@@ -1632,8 +2067,14 @@
       <c r="F31" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G31" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="H31" s="8" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="49.95" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>56</v>
       </c>
@@ -1652,8 +2093,14 @@
       <c r="F32" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G32" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="H32" s="8" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="49.95" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>57</v>
       </c>
@@ -1672,8 +2119,14 @@
       <c r="F33" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G33" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="H33" s="8" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="49.95" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>58</v>
       </c>
@@ -1692,8 +2145,14 @@
       <c r="F34" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G34" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="H34" s="8" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="49.95" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>59</v>
       </c>
@@ -1712,8 +2171,14 @@
       <c r="F35" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G35" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="49.95" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>60</v>
       </c>
@@ -1732,8 +2197,14 @@
       <c r="F36" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G36" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="49.95" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>61</v>
       </c>
@@ -1752,8 +2223,14 @@
       <c r="F37" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G37" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="H37" s="8" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="49.95" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>64</v>
       </c>
@@ -1772,8 +2249,14 @@
       <c r="F38" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G38" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="49.95" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>65</v>
       </c>
@@ -1792,8 +2275,14 @@
       <c r="F39" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G39" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="H39" s="8" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="49.95" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>68</v>
       </c>
@@ -1812,8 +2301,14 @@
       <c r="F40" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G40" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="49.95" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>69</v>
       </c>
@@ -1832,8 +2327,14 @@
       <c r="F41" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G41" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="H41" s="8" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="49.95" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>72</v>
       </c>
@@ -1852,8 +2353,14 @@
       <c r="F42" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G42" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="H42" s="8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="49.95" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>73</v>
       </c>
@@ -1872,8 +2379,14 @@
       <c r="F43" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G43" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="H43" s="8" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="49.95" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>74</v>
       </c>
@@ -1892,8 +2405,14 @@
       <c r="F44" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G44" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="H44" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="49.95" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>75</v>
       </c>
@@ -1912,8 +2431,14 @@
       <c r="F45" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G45" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="H45" s="8" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="49.95" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>78</v>
       </c>
@@ -1932,8 +2457,14 @@
       <c r="F46" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G46" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="H46" s="8" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="49.95" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>82</v>
       </c>
@@ -1952,8 +2483,14 @@
       <c r="F47" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G47" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="H47" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="49.95" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>85</v>
       </c>
@@ -1972,8 +2509,14 @@
       <c r="F48" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G48" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="H48" s="8" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="49.95" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>86</v>
       </c>
@@ -1992,8 +2535,14 @@
       <c r="F49" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="61.2" customHeight="1">
+      <c r="G49" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="H49" s="8" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="61.2" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>87</v>
       </c>
@@ -2012,8 +2561,14 @@
       <c r="F50" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="49.95" customHeight="1">
+      <c r="G50" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="H50" s="8" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="49.95" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>88</v>
       </c>
@@ -2031,6 +2586,12 @@
       </c>
       <c r="F51" s="3" t="s">
         <v>11</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="H51" s="8" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update test cases spreadsheet with modified test scenarios
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/274008f7bd52386a/Desktop/IT23377158/test_automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{6093456D-2646-4D6B-8FF5-3CCDE59B9837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F48009F8-F73F-4E28-8756-AFC3AFFE6BDD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF766E5-294D-4441-ADE1-8BCA0E4494D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,9 +46,6 @@
     <t>S</t>
   </si>
   <si>
-    <t>ඔයා ගෙදර යනවද?</t>
-  </si>
-  <si>
     <t>Neg_0002</t>
   </si>
   <si>
@@ -881,6 +878,9 @@
   </si>
   <si>
     <t>Evidence or rationale for the input type covered</t>
+  </si>
+  <si>
+    <t>ඇයි එහෙම කාරී?</t>
   </si>
 </sst>
 </file>
@@ -950,7 +950,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -961,12 +961,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1264,7 +1260,7 @@
     <col min="4" max="4" width="36.88671875" customWidth="1"/>
     <col min="5" max="5" width="71.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="104.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="104.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="46.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1287,11 +1283,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>286</v>
+      <c r="G1" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="49.95" customHeight="1">
@@ -1302,1296 +1298,1296 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="E2" s="3" t="s">
-        <v>104</v>
+        <v>286</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>236</v>
+        <v>10</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="49.95" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="F3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>237</v>
+        <v>10</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="49.95" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="F4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>238</v>
+        <v>10</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="58.8" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>109</v>
-      </c>
       <c r="F5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>239</v>
+        <v>10</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="49.95" customHeight="1">
       <c r="A6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="E6" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>240</v>
+        <v>10</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="49.95" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>112</v>
-      </c>
       <c r="F7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>241</v>
+        <v>10</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="49.95" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>115</v>
-      </c>
       <c r="F8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>242</v>
+        <v>10</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="49.95" customHeight="1">
       <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="E9" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>243</v>
+        <v>10</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="49.95" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>98</v>
-      </c>
       <c r="F10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>244</v>
+        <v>10</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="49.95" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="E11" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>245</v>
+        <v>10</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="49.95" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>148</v>
-      </c>
       <c r="F12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>246</v>
+        <v>10</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="49.95" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>130</v>
-      </c>
       <c r="F13" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>247</v>
+        <v>10</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="49.95" customHeight="1">
       <c r="A14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="E14" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>248</v>
+        <v>10</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="49.95" customHeight="1">
       <c r="A15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>30</v>
-      </c>
       <c r="F15" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>249</v>
+        <v>10</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="49.95" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="F16" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>250</v>
+        <v>10</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="49.95" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>151</v>
-      </c>
       <c r="F17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>251</v>
+        <v>10</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="49.95" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>154</v>
-      </c>
       <c r="F18" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>252</v>
+        <v>10</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="49.95" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>186</v>
-      </c>
       <c r="F19" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>253</v>
+        <v>10</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="49.95" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>157</v>
-      </c>
       <c r="F20" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>254</v>
+        <v>10</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="49.95" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="F21" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>255</v>
+        <v>10</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="49.95" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>160</v>
-      </c>
       <c r="F22" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G22" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>256</v>
+        <v>10</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="49.95" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>199</v>
-      </c>
       <c r="E23" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>257</v>
+        <v>10</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="49.95" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>163</v>
-      </c>
       <c r="F24" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>258</v>
+        <v>10</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="49.95" customHeight="1">
       <c r="A25" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="C25" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="E25" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="E25" s="3" t="s">
-        <v>196</v>
-      </c>
       <c r="F25" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>259</v>
+        <v>10</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="49.95" customHeight="1">
       <c r="A26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>260</v>
+        <v>10</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="49.95" customHeight="1">
       <c r="A27" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="E27" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>261</v>
+        <v>10</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="49.95" customHeight="1">
       <c r="A28" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="E28" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>262</v>
+        <v>10</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="49.95" customHeight="1">
       <c r="A29" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="E29" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="H29" s="8" t="s">
-        <v>263</v>
+        <v>10</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="49.95" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>188</v>
-      </c>
       <c r="F30" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="H30" s="8" t="s">
-        <v>264</v>
+        <v>10</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="49.95" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="E31" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="E31" s="3" t="s">
-        <v>202</v>
-      </c>
       <c r="F31" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="H31" s="8" t="s">
-        <v>265</v>
+        <v>10</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="49.95" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="F32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>266</v>
+        <v>10</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="49.95" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="E33" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="E33" s="3" t="s">
-        <v>193</v>
-      </c>
       <c r="F33" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="H33" s="8" t="s">
-        <v>267</v>
+        <v>10</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="49.95" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C34" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>204</v>
-      </c>
       <c r="F34" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G34" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="H34" s="8" t="s">
-        <v>268</v>
+        <v>10</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="49.95" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="E35" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="E35" s="3" t="s">
-        <v>208</v>
-      </c>
       <c r="F35" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>269</v>
+        <v>10</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="49.95" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>181</v>
-      </c>
       <c r="F36" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G36" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="H36" s="8" t="s">
-        <v>270</v>
+        <v>10</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="49.95" customHeight="1">
       <c r="A37" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E37" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>63</v>
-      </c>
       <c r="F37" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G37" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="H37" s="8" t="s">
-        <v>271</v>
+        <v>10</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="49.95" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C38" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>176</v>
-      </c>
       <c r="E38" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G38" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="H38" s="8" t="s">
-        <v>272</v>
+        <v>10</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="49.95" customHeight="1">
       <c r="A39" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="E39" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="H39" s="8" t="s">
-        <v>273</v>
+        <v>10</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="49.95" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="E40" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E40" s="3" t="s">
-        <v>173</v>
-      </c>
       <c r="F40" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G40" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="H40" s="8" t="s">
-        <v>274</v>
+        <v>10</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="49.95" customHeight="1">
       <c r="A41" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="E41" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="H41" s="8" t="s">
-        <v>275</v>
+        <v>10</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="49.95" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>140</v>
-      </c>
       <c r="E42" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G42" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="H42" s="8" t="s">
-        <v>276</v>
+        <v>10</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="49.95" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="F43" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G43" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="H43" s="8" t="s">
-        <v>277</v>
+        <v>10</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="49.95" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E44" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>170</v>
-      </c>
       <c r="F44" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G44" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="H44" s="8" t="s">
-        <v>278</v>
+        <v>10</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="49.95" customHeight="1">
       <c r="A45" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="E45" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G45" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="H45" s="8" t="s">
-        <v>279</v>
+        <v>10</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="49.95" customHeight="1">
       <c r="A46" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="E46" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G46" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="H46" s="8" t="s">
-        <v>280</v>
+        <v>10</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="49.95" customHeight="1">
       <c r="A47" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C47" s="2" t="s">
+      <c r="D47" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="E47" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G47" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="H47" s="8" t="s">
-        <v>281</v>
+        <v>10</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="49.95" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>133</v>
-      </c>
       <c r="F48" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="H48" s="8" t="s">
-        <v>282</v>
+        <v>10</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="49.95" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C49" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E49" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>136</v>
-      </c>
       <c r="F49" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G49" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="H49" s="8" t="s">
-        <v>283</v>
+        <v>10</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="61.2" customHeight="1">
       <c r="A50" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>166</v>
-      </c>
       <c r="F50" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="H50" s="8" t="s">
-        <v>284</v>
+        <v>10</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="49.95" customHeight="1">
       <c r="A51" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C51" s="2" t="s">
+      <c r="D51" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D51" s="2" t="s">
-        <v>90</v>
-      </c>
       <c r="E51" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="H51" s="8" t="s">
-        <v>285</v>
+        <v>10</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>